<commit_message>
Update Groq-planned Bosch benchmark results
</commit_message>
<xml_diff>
--- a/output/bosch_plasma_etch/bosch_benchmark_report.xlsx
+++ b/output/bosch_plasma_etch/bosch_benchmark_report.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Top_3_Models" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Wafer_Average_Si_Etch" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Map_Point_Si_Etch" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="All_Metrics" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top_3_Models" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wafer_Average_Si_Etch" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Map_Point_Si_Etch" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All_Metrics" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -528,7 +528,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Lasso (R² = 0.8837, RMSE = 0.1363)</t>
+          <t>Lightgbm (R² = 0.7874, RMSE = 0.1843)</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Lightgbm (R² = 0.9925)</t>
+          <t>Random Forest (R² = 0.9900)</t>
         </is>
       </c>
     </row>
@@ -606,22 +606,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Regularised Linear</t>
+          <t>Boosting Ensemble</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lasso</t>
+          <t>Lightgbm</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.8837</v>
+        <v>0.7874</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1363</v>
+        <v>0.1843</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1091</v>
+        <v>0.1527</v>
       </c>
       <c r="G2" t="n">
         <v>88</v>
@@ -636,22 +636,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Regularised Linear</t>
+          <t>Boosting Ensemble</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Elastic Net</t>
+          <t>Xgboost</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.8834</v>
+        <v>0.7852</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1364</v>
+        <v>0.1852</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1096</v>
+        <v>0.1569</v>
       </c>
       <c r="G3" t="n">
         <v>88</v>
@@ -671,17 +671,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Lightgbm</t>
+          <t>Hist Gradient Boosting</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.8324</v>
+        <v>0.7496</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1636</v>
+        <v>0.2</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1291</v>
+        <v>0.1598</v>
       </c>
       <c r="G4" t="n">
         <v>88</v>
@@ -752,22 +752,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Regularised Linear</t>
+          <t>Boosting Ensemble</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lasso</t>
+          <t>Lightgbm</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.8837</v>
+        <v>0.7874</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1363</v>
+        <v>0.1843</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1091</v>
+        <v>0.1527</v>
       </c>
       <c r="G2" t="n">
         <v>88</v>
@@ -782,22 +782,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Regularised Linear</t>
+          <t>Boosting Ensemble</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Elastic Net</t>
+          <t>Xgboost</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.8834</v>
+        <v>0.7852</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1364</v>
+        <v>0.1852</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1096</v>
+        <v>0.1569</v>
       </c>
       <c r="G3" t="n">
         <v>88</v>
@@ -817,17 +817,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Lightgbm</t>
+          <t>Hist Gradient Boosting</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.8324</v>
+        <v>0.7496</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1636</v>
+        <v>0.2</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1291</v>
+        <v>0.1598</v>
       </c>
       <c r="G4" t="n">
         <v>88</v>
@@ -842,22 +842,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Boosting Ensemble</t>
+          <t>Regularised Linear</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Xgboost</t>
+          <t>Elastic Net</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.8323</v>
+        <v>0.7485000000000001</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1636</v>
+        <v>0.2004</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1351</v>
+        <v>0.1564</v>
       </c>
       <c r="G5" t="n">
         <v>88</v>
@@ -872,22 +872,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bagging Ensemble</t>
+          <t>Regularised Linear</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Extra Trees</t>
+          <t>Lasso</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.7958</v>
+        <v>0.7351</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1806</v>
+        <v>0.2057</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1471</v>
+        <v>0.1682</v>
       </c>
       <c r="G6" t="n">
         <v>88</v>
@@ -902,22 +902,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Boosting Ensemble</t>
+          <t>Bagging Ensemble</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Hist Gradient Boosting</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.7703</v>
+        <v>0.7279</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1915</v>
+        <v>0.2085</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1626</v>
+        <v>0.171</v>
       </c>
       <c r="G7" t="n">
         <v>88</v>
@@ -941,13 +941,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.7467</v>
+        <v>0.6969</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2011</v>
+        <v>0.22</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1702</v>
+        <v>0.1811</v>
       </c>
       <c r="G8" t="n">
         <v>88</v>
@@ -971,13 +971,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.6221</v>
+        <v>0.5382</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2457</v>
+        <v>0.2716</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2037</v>
+        <v>0.2253</v>
       </c>
       <c r="G9" t="n">
         <v>88</v>
@@ -1031,13 +1031,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>-3.2184</v>
+        <v>-53.2402</v>
       </c>
       <c r="E11" t="n">
-        <v>0.8208</v>
+        <v>2.9431</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1962</v>
+        <v>0.4746</v>
       </c>
       <c r="G11" t="n">
         <v>88</v>
@@ -1113,12 +1113,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Boosting Ensemble</t>
+          <t>Bagging Ensemble</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lightgbm</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1127,13 +1127,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.9925</v>
+        <v>0.99</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3135</v>
+        <v>0.3602</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1677</v>
+        <v>0.2257</v>
       </c>
       <c r="H2" t="n">
         <v>7832</v>
@@ -1153,7 +1153,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Xgboost</t>
+          <t>Lightgbm</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1162,13 +1162,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.9921</v>
+        <v>0.99</v>
       </c>
       <c r="F3" t="n">
-        <v>0.321</v>
+        <v>0.3607</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1739</v>
+        <v>0.2204</v>
       </c>
       <c r="H3" t="n">
         <v>7832</v>
@@ -1183,12 +1183,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Boosting Ensemble</t>
+          <t>Bagging Ensemble</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hist Gradient Boosting</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1197,13 +1197,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.9921</v>
+        <v>0.99</v>
       </c>
       <c r="F4" t="n">
-        <v>0.3218</v>
+        <v>0.3616</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1766</v>
+        <v>0.2271</v>
       </c>
       <c r="H4" t="n">
         <v>7832</v>
@@ -1218,12 +1218,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bagging Ensemble</t>
+          <t>Boosting Ensemble</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Extra Trees</t>
+          <t>Hist Gradient Boosting</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1232,13 +1232,13 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.9913999999999999</v>
+        <v>0.9896</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3351</v>
+        <v>0.3675</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1844</v>
+        <v>0.231</v>
       </c>
       <c r="H5" t="n">
         <v>7832</v>
@@ -1253,12 +1253,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bagging Ensemble</t>
+          <t>Boosting Ensemble</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>Xgboost</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1267,13 +1267,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.991</v>
+        <v>0.9868</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3421</v>
+        <v>0.4148</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1948</v>
+        <v>0.2797</v>
       </c>
       <c r="H6" t="n">
         <v>7832</v>
@@ -1302,13 +1302,13 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.9044</v>
+        <v>0.9031</v>
       </c>
       <c r="F7" t="n">
-        <v>1.1159</v>
+        <v>1.1234</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9334</v>
+        <v>0.9386</v>
       </c>
       <c r="H7" t="n">
         <v>7832</v>
@@ -1337,13 +1337,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.8949</v>
+        <v>0.8937</v>
       </c>
       <c r="F8" t="n">
-        <v>1.1705</v>
+        <v>1.1769</v>
       </c>
       <c r="G8" t="n">
-        <v>1.0176</v>
+        <v>1.0198</v>
       </c>
       <c r="H8" t="n">
         <v>7832</v>
@@ -1372,13 +1372,13 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.8384</v>
+        <v>0.7955</v>
       </c>
       <c r="F9" t="n">
-        <v>1.451</v>
+        <v>1.6324</v>
       </c>
       <c r="G9" t="n">
-        <v>0.9106</v>
+        <v>1.0882</v>
       </c>
       <c r="H9" t="n">
         <v>7832</v>
@@ -1407,13 +1407,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.5805</v>
+        <v>0.7933</v>
       </c>
       <c r="F10" t="n">
-        <v>2.3379</v>
+        <v>1.6413</v>
       </c>
       <c r="G10" t="n">
-        <v>1.1712</v>
+        <v>1.085</v>
       </c>
       <c r="H10" t="n">
         <v>7832</v>
@@ -1536,7 +1536,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>coordinate_only</t>
+          <t>process_plus_coordinate</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1551,13 +1551,13 @@
         <v>10</v>
       </c>
       <c r="G2" t="n">
-        <v>0.05901200967723907</v>
+        <v>0.1023097095939609</v>
       </c>
       <c r="H2" t="n">
-        <v>0.07499181666119883</v>
+        <v>0.07324619991789533</v>
       </c>
       <c r="I2" t="n">
-        <v>0.05156047208512177</v>
+        <v>0.05282534372258398</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>process_only</t>
+          <t>coordinate_only</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1593,13 +1593,13 @@
         <v>10</v>
       </c>
       <c r="G3" t="n">
-        <v>0.00526969437827951</v>
+        <v>0.05908355951480637</v>
       </c>
       <c r="H3" t="n">
-        <v>0.07710357388458154</v>
+        <v>0.07498896553325833</v>
       </c>
       <c r="I3" t="n">
-        <v>0.05961422145681942</v>
+        <v>0.05167555365762547</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>process_plus_coordinate</t>
+          <t>process_only</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1635,13 +1635,13 @@
         <v>10</v>
       </c>
       <c r="G4" t="n">
-        <v>0.001877880564245205</v>
+        <v>0.04141248636057648</v>
       </c>
       <c r="H4" t="n">
-        <v>0.07723491522022354</v>
+        <v>0.07568986278728099</v>
       </c>
       <c r="I4" t="n">
-        <v>0.05708877687555702</v>
+        <v>0.05854347954439177</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>process_only</t>
+          <t>coordinate_only</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1677,13 +1677,13 @@
         <v>10</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.01894953462408266</v>
+        <v>-0.04626465837118143</v>
       </c>
       <c r="H5" t="n">
-        <v>0.07803656990694241</v>
+        <v>0.07907562112400479</v>
       </c>
       <c r="I5" t="n">
-        <v>0.06161416033970223</v>
+        <v>0.05792354298041798</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ridge</t>
+          <t>dummy_mean</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1719,17 +1719,17 @@
         <v>10</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.04626465837118143</v>
+        <v>-0.05351699029592072</v>
       </c>
       <c r="H6" t="n">
-        <v>0.07907562112400479</v>
+        <v>0.07934920978168188</v>
       </c>
       <c r="I6" t="n">
-        <v>0.05792354298041798</v>
+        <v>0.06130529082337945</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Regularised Linear</t>
+          <t>Baseline</t>
         </is>
       </c>
     </row>
@@ -1746,12 +1746,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>process_plus_coordinate</t>
+          <t>process_only</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ridge</t>
+          <t>dummy_mean</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1761,17 +1761,17 @@
         <v>10</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.05049515807542693</v>
+        <v>-0.05351699029592072</v>
       </c>
       <c r="H7" t="n">
-        <v>0.07923532828287706</v>
+        <v>0.07934920978168188</v>
       </c>
       <c r="I7" t="n">
-        <v>0.06322737795236327</v>
+        <v>0.06130529082337945</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Regularised Linear</t>
+          <t>Baseline</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>coordinate_only</t>
+          <t>process_plus_coordinate</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>dummy_mean</t>
+          <t>ridge</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1845,17 +1845,17 @@
         <v>10</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.05351699029592072</v>
+        <v>-22.48799129895567</v>
       </c>
       <c r="H9" t="n">
-        <v>0.07934920978168188</v>
+        <v>0.3746664218907106</v>
       </c>
       <c r="I9" t="n">
-        <v>0.06130529082337945</v>
+        <v>0.09632784806758846</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Baseline</t>
+          <t>Regularised Linear</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1877,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>dummy_mean</t>
+          <t>ridge</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -1887,17 +1887,17 @@
         <v>10</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.05351699029592072</v>
+        <v>-22.49503788000173</v>
       </c>
       <c r="H10" t="n">
-        <v>0.07934920978168188</v>
+        <v>0.3747226191041979</v>
       </c>
       <c r="I10" t="n">
-        <v>0.06130529082337945</v>
+        <v>0.09682020776509064</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Baseline</t>
+          <t>Regularised Linear</t>
         </is>
       </c>
     </row>
@@ -1919,7 +1919,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>lightgbm</t>
+          <t>random_forest</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -1929,17 +1929,17 @@
         <v>10</v>
       </c>
       <c r="G11" t="n">
-        <v>0.9924577011546956</v>
+        <v>0.9900425925136996</v>
       </c>
       <c r="H11" t="n">
-        <v>0.3134898524702177</v>
+        <v>0.3602008716058591</v>
       </c>
       <c r="I11" t="n">
-        <v>0.1677114105805036</v>
+        <v>0.2256532735648406</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Boosting Ensemble</t>
+          <t>Bagging Ensemble</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>lightgbm</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -1971,13 +1971,13 @@
         <v>10</v>
       </c>
       <c r="G12" t="n">
-        <v>0.9920939740671423</v>
+        <v>0.9900138975313226</v>
       </c>
       <c r="H12" t="n">
-        <v>0.3209598708682734</v>
+        <v>0.360719506698272</v>
       </c>
       <c r="I12" t="n">
-        <v>0.1738882198906928</v>
+        <v>0.2204220380654019</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>hist_gradient_boosting</t>
+          <t>extra_trees</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -2013,17 +2013,17 @@
         <v>10</v>
       </c>
       <c r="G13" t="n">
-        <v>0.9920507716961628</v>
+        <v>0.9899658780771068</v>
       </c>
       <c r="H13" t="n">
-        <v>0.3218356165435544</v>
+        <v>0.3615857495882452</v>
       </c>
       <c r="I13" t="n">
-        <v>0.1765516991045911</v>
+        <v>0.2270617471379432</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Boosting Ensemble</t>
+          <t>Bagging Ensemble</t>
         </is>
       </c>
     </row>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>extra_trees</t>
+          <t>hist_gradient_boosting</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -2055,17 +2055,17 @@
         <v>10</v>
       </c>
       <c r="G14" t="n">
-        <v>0.9913834509468943</v>
+        <v>0.9896337006640433</v>
       </c>
       <c r="H14" t="n">
-        <v>0.3350721263740687</v>
+        <v>0.367522127588029</v>
       </c>
       <c r="I14" t="n">
-        <v>0.1843735022002269</v>
+        <v>0.2310105264329834</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Bagging Ensemble</t>
+          <t>Boosting Ensemble</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -2097,17 +2097,17 @@
         <v>10</v>
       </c>
       <c r="G15" t="n">
-        <v>0.9910171041368855</v>
+        <v>0.9867950650619893</v>
       </c>
       <c r="H15" t="n">
-        <v>0.3421210544089624</v>
+        <v>0.4148009593969081</v>
       </c>
       <c r="I15" t="n">
-        <v>0.1948312250268316</v>
+        <v>0.2796658573585904</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Bagging Ensemble</t>
+          <t>Boosting Ensemble</t>
         </is>
       </c>
     </row>
@@ -2139,13 +2139,13 @@
         <v>10</v>
       </c>
       <c r="G16" t="n">
-        <v>0.9818921174435982</v>
+        <v>0.9818353188357193</v>
       </c>
       <c r="H16" t="n">
-        <v>0.4857417732078295</v>
+        <v>0.4865029846711463</v>
       </c>
       <c r="I16" t="n">
-        <v>0.3608876451611659</v>
+        <v>0.3614266482057837</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -2181,13 +2181,13 @@
         <v>10</v>
       </c>
       <c r="G17" t="n">
-        <v>0.9044279326701293</v>
+        <v>0.9031364980164232</v>
       </c>
       <c r="H17" t="n">
-        <v>1.115930402053991</v>
+        <v>1.123444707210731</v>
       </c>
       <c r="I17" t="n">
-        <v>0.9333572840267329</v>
+        <v>0.9385901230540494</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -2223,13 +2223,13 @@
         <v>10</v>
       </c>
       <c r="G18" t="n">
-        <v>0.894853478288587</v>
+        <v>0.8936927006283796</v>
       </c>
       <c r="H18" t="n">
-        <v>1.170493684178947</v>
+        <v>1.176936853286116</v>
       </c>
       <c r="I18" t="n">
-        <v>1.017604346018256</v>
+        <v>1.019844219268593</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -2307,13 +2307,13 @@
         <v>10</v>
       </c>
       <c r="G20" t="n">
-        <v>0.8384226113944081</v>
+        <v>0.7955024339056359</v>
       </c>
       <c r="H20" t="n">
-        <v>1.45098162204284</v>
+        <v>1.63235904888604</v>
       </c>
       <c r="I20" t="n">
-        <v>0.9106255123541714</v>
+        <v>1.088240197693519</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -2349,13 +2349,13 @@
         <v>10</v>
       </c>
       <c r="G21" t="n">
-        <v>0.5805259661160509</v>
+        <v>0.7932522455593631</v>
       </c>
       <c r="H21" t="n">
-        <v>2.337890469631078</v>
+        <v>1.641315307662666</v>
       </c>
       <c r="I21" t="n">
-        <v>1.171214771280065</v>
+        <v>1.085020524150531</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -2391,13 +2391,13 @@
         <v>10</v>
       </c>
       <c r="G22" t="n">
-        <v>0.009816361887350467</v>
+        <v>0.009326139638412334</v>
       </c>
       <c r="H22" t="n">
-        <v>3.59194346235671</v>
+        <v>3.592832505887078</v>
       </c>
       <c r="I22" t="n">
-        <v>2.969348308530383</v>
+        <v>2.969360461736378</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -2559,13 +2559,13 @@
         <v>10</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.3046001327563272</v>
+        <v>-8.251864495870906</v>
       </c>
       <c r="H26" t="n">
-        <v>4.122971459822725</v>
+        <v>10.97959323728449</v>
       </c>
       <c r="I26" t="n">
-        <v>3.15172086691683</v>
+        <v>4.033420382605369</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>ridge</t>
+          <t>extra_trees</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -2601,17 +2601,17 @@
         <v>10</v>
       </c>
       <c r="G27" t="n">
-        <v>0.4318597584142744</v>
+        <v>0.1020256562865285</v>
       </c>
       <c r="H27" t="n">
-        <v>0.03270628214311949</v>
+        <v>0.04111832049858792</v>
       </c>
       <c r="I27" t="n">
-        <v>0.02511777081936829</v>
+        <v>0.03228489790060225</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Regularised Linear</t>
+          <t>Bagging Ensemble</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2633,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>extra_trees</t>
+          <t>dummy_mean</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -2643,17 +2643,17 @@
         <v>10</v>
       </c>
       <c r="G28" t="n">
-        <v>0.05032494181718683</v>
+        <v>-0.1698746376933444</v>
       </c>
       <c r="H28" t="n">
-        <v>0.04228544634151089</v>
+        <v>0.04693243269279635</v>
       </c>
       <c r="I28" t="n">
-        <v>0.03337700870723784</v>
+        <v>0.03956008478033084</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Bagging Ensemble</t>
+          <t>Baseline</t>
         </is>
       </c>
     </row>
@@ -2675,7 +2675,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>dummy_mean</t>
+          <t>ridge</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -2685,17 +2685,17 @@
         <v>10</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.1698746376933444</v>
+        <v>-2.719547656485952</v>
       </c>
       <c r="H29" t="n">
-        <v>0.04693243269279635</v>
+        <v>0.08368516308624657</v>
       </c>
       <c r="I29" t="n">
-        <v>0.03956008478033084</v>
+        <v>0.03147311300790716</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Baseline</t>
+          <t>Regularised Linear</t>
         </is>
       </c>
     </row>
@@ -2717,7 +2717,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>lasso</t>
+          <t>lightgbm</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -2727,17 +2727,17 @@
         <v>10</v>
       </c>
       <c r="G30" t="n">
-        <v>0.8837373463060553</v>
+        <v>0.7874044625738486</v>
       </c>
       <c r="H30" t="n">
-        <v>0.1362592106627554</v>
+        <v>0.1842565032609901</v>
       </c>
       <c r="I30" t="n">
-        <v>0.1091233564101</v>
+        <v>0.1527160324888304</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Regularised Linear</t>
+          <t>Boosting Ensemble</t>
         </is>
       </c>
     </row>
@@ -2759,7 +2759,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>elastic_net</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -2769,17 +2769,17 @@
         <v>10</v>
       </c>
       <c r="G31" t="n">
-        <v>0.8834401263177255</v>
+        <v>0.7852041072962006</v>
       </c>
       <c r="H31" t="n">
-        <v>0.136433269611732</v>
+        <v>0.1852075724197131</v>
       </c>
       <c r="I31" t="n">
-        <v>0.1096127434612005</v>
+        <v>0.156926080692631</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Regularised Linear</t>
+          <t>Boosting Ensemble</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>lightgbm</t>
+          <t>hist_gradient_boosting</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -2811,13 +2811,13 @@
         <v>10</v>
       </c>
       <c r="G32" t="n">
-        <v>0.8323502544096504</v>
+        <v>0.7496278471301723</v>
       </c>
       <c r="H32" t="n">
-        <v>0.1636240742392344</v>
+        <v>0.1999579910868704</v>
       </c>
       <c r="I32" t="n">
-        <v>0.1290772160339037</v>
+        <v>0.1597913478676823</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -2843,7 +2843,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>elastic_net</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -2853,17 +2853,17 @@
         <v>10</v>
       </c>
       <c r="G33" t="n">
-        <v>0.8323269763578304</v>
+        <v>0.7485464360303347</v>
       </c>
       <c r="H33" t="n">
-        <v>0.163635433390007</v>
+        <v>0.2003893565526343</v>
       </c>
       <c r="I33" t="n">
-        <v>0.135127981808769</v>
+        <v>0.1564375473073731</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Boosting Ensemble</t>
+          <t>Regularised Linear</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>extra_trees</t>
+          <t>lasso</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -2895,17 +2895,17 @@
         <v>10</v>
       </c>
       <c r="G34" t="n">
-        <v>0.7958135674948011</v>
+        <v>0.735093540751985</v>
       </c>
       <c r="H34" t="n">
-        <v>0.1805756528559495</v>
+        <v>0.2056799826374968</v>
       </c>
       <c r="I34" t="n">
-        <v>0.1471155265138497</v>
+        <v>0.1682332566819065</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Bagging Ensemble</t>
+          <t>Regularised Linear</t>
         </is>
       </c>
     </row>
@@ -2927,7 +2927,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>hist_gradient_boosting</t>
+          <t>extra_trees</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -2937,17 +2937,17 @@
         <v>10</v>
       </c>
       <c r="G35" t="n">
-        <v>0.7702979041498136</v>
+        <v>0.727862529300543</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1915262175783858</v>
+        <v>0.2084682520903581</v>
       </c>
       <c r="I35" t="n">
-        <v>0.1625875718025192</v>
+        <v>0.1710265931812424</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Boosting Ensemble</t>
+          <t>Bagging Ensemble</t>
         </is>
       </c>
     </row>
@@ -2979,13 +2979,13 @@
         <v>10</v>
       </c>
       <c r="G36" t="n">
-        <v>0.7466661898282477</v>
+        <v>0.6969231002931857</v>
       </c>
       <c r="H36" t="n">
-        <v>0.2011371677894026</v>
+        <v>0.2199997417639609</v>
       </c>
       <c r="I36" t="n">
-        <v>0.1701993722003281</v>
+        <v>0.1810781908629178</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -3021,13 +3021,13 @@
         <v>10</v>
       </c>
       <c r="G37" t="n">
-        <v>0.6220918391473734</v>
+        <v>0.5382106896727945</v>
       </c>
       <c r="H37" t="n">
-        <v>0.2456625119542266</v>
+        <v>0.2715611822834366</v>
       </c>
       <c r="I37" t="n">
-        <v>0.2036616440168364</v>
+        <v>0.225274237417412</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -3105,13 +3105,13 @@
         <v>10</v>
       </c>
       <c r="G39" t="n">
-        <v>-3.218422716128226</v>
+        <v>-53.2402111151417</v>
       </c>
       <c r="H39" t="n">
-        <v>0.8207687288385354</v>
+        <v>2.943109622556281</v>
       </c>
       <c r="I39" t="n">
-        <v>0.1961985849573611</v>
+        <v>0.4745858376521649</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>

</xml_diff>